<commit_message>
Update HOTAS Switch and Button - Quick Reference - FULL.xlsx
Updated to include Mouse Emulation tweaks
</commit_message>
<xml_diff>
--- a/Maps/HOTAS Switch and Button - Quick Reference - FULL.xlsx
+++ b/Maps/HOTAS Switch and Button - Quick Reference - FULL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\Den\OneDrive\Personal\Thrustmaster\TARGET\Clicker\Development\ED_TargetScript-503\Maps\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B58D3CB5-21CC-4D9B-834B-C0205A49A2F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29FC7390-3705-407D-999A-74173DC06B71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2970" yWindow="660" windowWidth="28305" windowHeight="18765" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="690" yWindow="225" windowWidth="33450" windowHeight="18765" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="448" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="451" uniqueCount="242">
   <si>
     <t>TG1</t>
   </si>
@@ -742,6 +742,15 @@
   </si>
   <si>
     <t>HOTAS - Quick reference - v503 - FULL</t>
+  </si>
+  <si>
+    <t>Std FA-Off</t>
+  </si>
+  <si>
+    <t>tgMouseControl()</t>
+  </si>
+  <si>
+    <t>Mouse Mode for JS</t>
   </si>
 </sst>
 </file>
@@ -765,7 +774,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -790,6 +799,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="33">
     <border>
@@ -1233,7 +1248,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="68">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1364,71 +1379,77 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1758,24 +1779,24 @@
     </row>
     <row r="3" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B4" s="58" t="s">
+      <c r="B4" s="61" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="59"/>
-      <c r="D4" s="59"/>
-      <c r="E4" s="60"/>
-      <c r="G4" s="58" t="s">
+      <c r="C4" s="62"/>
+      <c r="D4" s="62"/>
+      <c r="E4" s="63"/>
+      <c r="G4" s="61" t="s">
         <v>202</v>
       </c>
-      <c r="H4" s="59"/>
-      <c r="I4" s="59"/>
-      <c r="J4" s="60"/>
-      <c r="L4" s="58" t="s">
+      <c r="H4" s="62"/>
+      <c r="I4" s="62"/>
+      <c r="J4" s="63"/>
+      <c r="L4" s="61" t="s">
         <v>49</v>
       </c>
-      <c r="M4" s="59"/>
-      <c r="N4" s="59"/>
-      <c r="O4" s="60"/>
+      <c r="M4" s="62"/>
+      <c r="N4" s="62"/>
+      <c r="O4" s="63"/>
     </row>
     <row r="5" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="8" t="s">
@@ -1817,7 +1838,7 @@
     </row>
     <row r="6" spans="2:15" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="7" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B7" s="48" t="s">
+      <c r="B7" s="47" t="s">
         <v>0</v>
       </c>
       <c r="C7" s="11" t="s">
@@ -1835,7 +1856,7 @@
         <v>115</v>
       </c>
       <c r="J7" s="18"/>
-      <c r="L7" s="48" t="s">
+      <c r="L7" s="47" t="s">
         <v>73</v>
       </c>
       <c r="M7" s="11" t="s">
@@ -1847,7 +1868,7 @@
       <c r="O7" s="12"/>
     </row>
     <row r="8" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="50"/>
+      <c r="B8" s="45"/>
       <c r="C8" s="2" t="s">
         <v>25</v>
       </c>
@@ -1865,7 +1886,7 @@
         <v>116</v>
       </c>
       <c r="J8" s="19"/>
-      <c r="L8" s="49"/>
+      <c r="L8" s="46"/>
       <c r="M8" s="4" t="s">
         <v>128</v>
       </c>
@@ -1875,7 +1896,7 @@
       <c r="O8" s="5"/>
     </row>
     <row r="9" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="49"/>
+      <c r="B9" s="46"/>
       <c r="C9" s="4" t="s">
         <v>26</v>
       </c>
@@ -1905,7 +1926,7 @@
       <c r="O9" s="36"/>
     </row>
     <row r="10" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="57" t="s">
+      <c r="B10" s="60" t="s">
         <v>2</v>
       </c>
       <c r="C10" s="6" t="s">
@@ -1913,7 +1934,7 @@
       </c>
       <c r="D10" s="6"/>
       <c r="E10" s="7"/>
-      <c r="L10" s="48" t="s">
+      <c r="L10" s="47" t="s">
         <v>75</v>
       </c>
       <c r="M10" s="11" t="s">
@@ -1925,13 +1946,13 @@
       <c r="O10" s="12"/>
     </row>
     <row r="11" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="57"/>
+      <c r="B11" s="60"/>
       <c r="C11" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D11" s="2"/>
       <c r="E11" s="21"/>
-      <c r="G11" s="51" t="s">
+      <c r="G11" s="57" t="s">
         <v>50</v>
       </c>
       <c r="H11" s="11" t="s">
@@ -1941,7 +1962,7 @@
         <v>52</v>
       </c>
       <c r="J11" s="12"/>
-      <c r="L11" s="49"/>
+      <c r="L11" s="46"/>
       <c r="M11" s="4" t="s">
         <v>128</v>
       </c>
@@ -1951,13 +1972,13 @@
       <c r="O11" s="5"/>
     </row>
     <row r="12" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="49"/>
+      <c r="B12" s="46"/>
       <c r="C12" s="22" t="s">
         <v>26</v>
       </c>
       <c r="D12" s="22"/>
       <c r="E12" s="5"/>
-      <c r="G12" s="52"/>
+      <c r="G12" s="58"/>
       <c r="H12" s="2" t="s">
         <v>25</v>
       </c>
@@ -1967,13 +1988,13 @@
       <c r="J12" s="3"/>
     </row>
     <row r="13" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G13" s="53"/>
+      <c r="G13" s="59"/>
       <c r="H13" s="4" t="s">
         <v>26</v>
       </c>
       <c r="I13" s="4"/>
       <c r="J13" s="5"/>
-      <c r="L13" s="48" t="s">
+      <c r="L13" s="47" t="s">
         <v>76</v>
       </c>
       <c r="M13" s="11" t="s">
@@ -1985,7 +2006,7 @@
       <c r="O13" s="12"/>
     </row>
     <row r="14" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="48" t="s">
+      <c r="B14" s="47" t="s">
         <v>27</v>
       </c>
       <c r="C14" s="11" t="s">
@@ -1996,7 +2017,7 @@
       </c>
       <c r="E14" s="12"/>
       <c r="G14" s="13"/>
-      <c r="L14" s="49"/>
+      <c r="L14" s="46"/>
       <c r="M14" s="4" t="s">
         <v>128</v>
       </c>
@@ -2006,7 +2027,7 @@
       <c r="O14" s="5"/>
     </row>
     <row r="15" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B15" s="50"/>
+      <c r="B15" s="45"/>
       <c r="C15" s="2" t="s">
         <v>25</v>
       </c>
@@ -2014,7 +2035,7 @@
         <v>4</v>
       </c>
       <c r="E15" s="3"/>
-      <c r="G15" s="51" t="s">
+      <c r="G15" s="57" t="s">
         <v>53</v>
       </c>
       <c r="H15" s="11" t="s">
@@ -2024,7 +2045,7 @@
         <v>161</v>
       </c>
       <c r="J15" s="12"/>
-      <c r="L15" s="50" t="s">
+      <c r="L15" s="45" t="s">
         <v>77</v>
       </c>
       <c r="M15" s="6"/>
@@ -2032,7 +2053,7 @@
       <c r="O15" s="7"/>
     </row>
     <row r="16" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="49"/>
+      <c r="B16" s="46"/>
       <c r="C16" s="4" t="s">
         <v>26</v>
       </c>
@@ -2040,7 +2061,7 @@
         <v>201</v>
       </c>
       <c r="E16" s="5"/>
-      <c r="G16" s="52"/>
+      <c r="G16" s="58"/>
       <c r="H16" s="2" t="s">
         <v>25</v>
       </c>
@@ -2048,7 +2069,7 @@
         <v>54</v>
       </c>
       <c r="J16" s="3"/>
-      <c r="L16" s="50"/>
+      <c r="L16" s="45"/>
       <c r="M16" s="2" t="s">
         <v>25</v>
       </c>
@@ -2059,19 +2080,19 @@
     </row>
     <row r="17" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B17" s="16"/>
-      <c r="G17" s="53"/>
+      <c r="G17" s="59"/>
       <c r="H17" s="4" t="s">
         <v>26</v>
       </c>
       <c r="I17" s="4"/>
       <c r="J17" s="5"/>
-      <c r="L17" s="49"/>
+      <c r="L17" s="46"/>
       <c r="M17" s="4"/>
       <c r="N17" s="4"/>
       <c r="O17" s="5"/>
     </row>
     <row r="18" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="48" t="s">
+      <c r="B18" s="47" t="s">
         <v>108</v>
       </c>
       <c r="C18" s="11" t="s">
@@ -2086,7 +2107,7 @@
       <c r="G18" s="13"/>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B19" s="50"/>
+      <c r="B19" s="45"/>
       <c r="C19" s="2" t="s">
         <v>25</v>
       </c>
@@ -2096,7 +2117,7 @@
       <c r="E19" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="G19" s="48" t="s">
+      <c r="G19" s="47" t="s">
         <v>55</v>
       </c>
       <c r="H19" s="11" t="s">
@@ -2106,7 +2127,7 @@
         <v>218</v>
       </c>
       <c r="J19" s="12"/>
-      <c r="L19" s="48" t="s">
+      <c r="L19" s="47" t="s">
         <v>78</v>
       </c>
       <c r="M19" s="11" t="s">
@@ -2118,7 +2139,7 @@
       <c r="O19" s="12"/>
     </row>
     <row r="20" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="49"/>
+      <c r="B20" s="46"/>
       <c r="C20" s="4" t="s">
         <v>26</v>
       </c>
@@ -2128,7 +2149,7 @@
       <c r="E20" s="5" t="s">
         <v>203</v>
       </c>
-      <c r="G20" s="47"/>
+      <c r="G20" s="48"/>
       <c r="H20" s="2" t="s">
         <v>128</v>
       </c>
@@ -2138,7 +2159,7 @@
       <c r="J20" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="L20" s="50"/>
+      <c r="L20" s="45"/>
       <c r="M20" s="2" t="s">
         <v>128</v>
       </c>
@@ -2147,7 +2168,7 @@
     </row>
     <row r="21" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B21" s="16"/>
-      <c r="G21" s="46" t="s">
+      <c r="G21" s="44" t="s">
         <v>56</v>
       </c>
       <c r="H21" s="2" t="s">
@@ -2157,7 +2178,7 @@
         <v>219</v>
       </c>
       <c r="J21" s="3"/>
-      <c r="L21" s="50"/>
+      <c r="L21" s="45"/>
       <c r="M21" s="2" t="s">
         <v>24</v>
       </c>
@@ -2173,7 +2194,7 @@
         <v>114</v>
       </c>
       <c r="E22" s="29"/>
-      <c r="G22" s="47"/>
+      <c r="G22" s="48"/>
       <c r="H22" s="2" t="s">
         <v>128</v>
       </c>
@@ -2183,7 +2204,7 @@
       <c r="J22" s="3" t="s">
         <v>165</v>
       </c>
-      <c r="L22" s="50"/>
+      <c r="L22" s="45"/>
       <c r="M22" s="2" t="s">
         <v>25</v>
       </c>
@@ -2193,7 +2214,7 @@
       <c r="O22" s="3"/>
     </row>
     <row r="23" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G23" s="46" t="s">
+      <c r="G23" s="44" t="s">
         <v>57</v>
       </c>
       <c r="H23" s="2" t="s">
@@ -2203,7 +2224,7 @@
         <v>220</v>
       </c>
       <c r="J23" s="3"/>
-      <c r="L23" s="49"/>
+      <c r="L23" s="46"/>
       <c r="M23" s="22" t="s">
         <v>26</v>
       </c>
@@ -2211,15 +2232,19 @@
       <c r="O23" s="5"/>
     </row>
     <row r="24" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B24" s="48" t="s">
+      <c r="B24" s="47" t="s">
         <v>28</v>
       </c>
       <c r="C24" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="D24" s="11"/>
-      <c r="E24" s="12"/>
-      <c r="G24" s="47"/>
+      <c r="D24" s="66" t="s">
+        <v>240</v>
+      </c>
+      <c r="E24" s="67" t="s">
+        <v>241</v>
+      </c>
+      <c r="G24" s="48"/>
       <c r="H24" s="2" t="s">
         <v>128</v>
       </c>
@@ -2227,7 +2252,7 @@
         <v>100</v>
       </c>
       <c r="J24" s="3"/>
-      <c r="L24" s="48" t="s">
+      <c r="L24" s="47" t="s">
         <v>79</v>
       </c>
       <c r="M24" s="11" t="s">
@@ -2237,15 +2262,17 @@
       <c r="O24" s="12"/>
     </row>
     <row r="25" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B25" s="50"/>
+      <c r="B25" s="45"/>
       <c r="C25" s="2" t="s">
         <v>25</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E25" s="3"/>
-      <c r="G25" s="46" t="s">
+      <c r="E25" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="G25" s="44" t="s">
         <v>58</v>
       </c>
       <c r="H25" s="2" t="s">
@@ -2255,7 +2282,7 @@
         <v>221</v>
       </c>
       <c r="J25" s="3"/>
-      <c r="L25" s="50"/>
+      <c r="L25" s="45"/>
       <c r="M25" s="2" t="s">
         <v>25</v>
       </c>
@@ -2265,13 +2292,13 @@
       <c r="O25" s="3"/>
     </row>
     <row r="26" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="49"/>
+      <c r="B26" s="46"/>
       <c r="C26" s="4" t="s">
         <v>26</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="5"/>
-      <c r="G26" s="49"/>
+      <c r="G26" s="46"/>
       <c r="H26" s="4" t="s">
         <v>128</v>
       </c>
@@ -2279,7 +2306,7 @@
         <v>101</v>
       </c>
       <c r="J26" s="5"/>
-      <c r="L26" s="49"/>
+      <c r="L26" s="46"/>
       <c r="M26" s="4" t="s">
         <v>26</v>
       </c>
@@ -2288,7 +2315,7 @@
     </row>
     <row r="27" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="28" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B28" s="48" t="s">
+      <c r="B28" s="47" t="s">
         <v>29</v>
       </c>
       <c r="C28" s="11" t="s">
@@ -2308,7 +2335,7 @@
       <c r="J28" s="12" t="s">
         <v>223</v>
       </c>
-      <c r="L28" s="48" t="s">
+      <c r="L28" s="47" t="s">
         <v>80</v>
       </c>
       <c r="M28" s="11" t="s">
@@ -2320,7 +2347,7 @@
       <c r="O28" s="12"/>
     </row>
     <row r="29" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="50"/>
+      <c r="B29" s="45"/>
       <c r="C29" s="2" t="s">
         <v>25</v>
       </c>
@@ -2338,7 +2365,7 @@
       <c r="J29" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="L29" s="49"/>
+      <c r="L29" s="46"/>
       <c r="M29" s="4" t="s">
         <v>128</v>
       </c>
@@ -2348,7 +2375,7 @@
       <c r="O29" s="5"/>
     </row>
     <row r="30" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="47"/>
+      <c r="B30" s="48"/>
       <c r="C30" s="2" t="s">
         <v>26</v>
       </c>
@@ -2368,7 +2395,7 @@
       </c>
     </row>
     <row r="31" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B31" s="46" t="s">
+      <c r="B31" s="44" t="s">
         <v>30</v>
       </c>
       <c r="C31" s="2" t="s">
@@ -2386,7 +2413,7 @@
       <c r="J31" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="L31" s="48" t="s">
+      <c r="L31" s="47" t="s">
         <v>81</v>
       </c>
       <c r="M31" s="11" t="s">
@@ -2398,7 +2425,7 @@
       <c r="O31" s="12"/>
     </row>
     <row r="32" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="50"/>
+      <c r="B32" s="45"/>
       <c r="C32" s="2" t="s">
         <v>25</v>
       </c>
@@ -2406,7 +2433,7 @@
         <v>7</v>
       </c>
       <c r="E32" s="3"/>
-      <c r="G32" s="46" t="s">
+      <c r="G32" s="44" t="s">
         <v>63</v>
       </c>
       <c r="H32" s="2" t="s">
@@ -2415,10 +2442,10 @@
       <c r="I32" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="J32" s="44" t="s">
+      <c r="J32" s="64" t="s">
         <v>223</v>
       </c>
-      <c r="L32" s="49"/>
+      <c r="L32" s="46"/>
       <c r="M32" s="4" t="s">
         <v>128</v>
       </c>
@@ -2428,23 +2455,23 @@
       <c r="O32" s="5"/>
     </row>
     <row r="33" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="47"/>
+      <c r="B33" s="48"/>
       <c r="C33" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="3"/>
-      <c r="G33" s="47"/>
+      <c r="G33" s="48"/>
       <c r="H33" s="2" t="s">
         <v>128</v>
       </c>
       <c r="I33" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="J33" s="45"/>
+      <c r="J33" s="65"/>
     </row>
     <row r="34" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="46" t="s">
+      <c r="B34" s="44" t="s">
         <v>31</v>
       </c>
       <c r="C34" s="2" t="s">
@@ -2462,7 +2489,7 @@
       <c r="J34" s="3" t="s">
         <v>223</v>
       </c>
-      <c r="L34" s="48" t="s">
+      <c r="L34" s="47" t="s">
         <v>82</v>
       </c>
       <c r="M34" s="11" t="s">
@@ -2474,7 +2501,7 @@
       <c r="O34" s="12"/>
     </row>
     <row r="35" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="50"/>
+      <c r="B35" s="45"/>
       <c r="C35" s="2" t="s">
         <v>25</v>
       </c>
@@ -2484,7 +2511,7 @@
       <c r="E35" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="L35" s="50"/>
+      <c r="L35" s="45"/>
       <c r="M35" s="2" t="s">
         <v>25</v>
       </c>
@@ -2496,13 +2523,13 @@
       </c>
     </row>
     <row r="36" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B36" s="47"/>
+      <c r="B36" s="48"/>
       <c r="C36" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D36" s="2"/>
       <c r="E36" s="3"/>
-      <c r="G36" s="48" t="s">
+      <c r="G36" s="47" t="s">
         <v>64</v>
       </c>
       <c r="H36" s="11" t="s">
@@ -2514,7 +2541,7 @@
       <c r="J36" s="12" t="s">
         <v>166</v>
       </c>
-      <c r="L36" s="47"/>
+      <c r="L36" s="48"/>
       <c r="M36" s="2" t="s">
         <v>26</v>
       </c>
@@ -2524,7 +2551,7 @@
       <c r="O36" s="3"/>
     </row>
     <row r="37" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B37" s="46" t="s">
+      <c r="B37" s="44" t="s">
         <v>32</v>
       </c>
       <c r="C37" s="2" t="s">
@@ -2536,7 +2563,7 @@
       <c r="E37" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="G37" s="50"/>
+      <c r="G37" s="45"/>
       <c r="H37" s="2" t="s">
         <v>25</v>
       </c>
@@ -2546,7 +2573,7 @@
       <c r="J37" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="L37" s="46" t="s">
+      <c r="L37" s="44" t="s">
         <v>181</v>
       </c>
       <c r="M37" s="2" t="s">
@@ -2556,7 +2583,7 @@
       <c r="O37" s="3"/>
     </row>
     <row r="38" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B38" s="50"/>
+      <c r="B38" s="45"/>
       <c r="C38" s="2" t="s">
         <v>25</v>
       </c>
@@ -2566,7 +2593,7 @@
       <c r="E38" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="G38" s="47"/>
+      <c r="G38" s="48"/>
       <c r="H38" s="2" t="s">
         <v>26</v>
       </c>
@@ -2576,7 +2603,7 @@
       <c r="J38" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="L38" s="50"/>
+      <c r="L38" s="45"/>
       <c r="M38" s="2" t="s">
         <v>25</v>
       </c>
@@ -2588,7 +2615,7 @@
       </c>
     </row>
     <row r="39" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="49"/>
+      <c r="B39" s="46"/>
       <c r="C39" s="4" t="s">
         <v>26</v>
       </c>
@@ -2604,7 +2631,7 @@
       <c r="J39" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="L39" s="47"/>
+      <c r="L39" s="48"/>
       <c r="M39" s="2" t="s">
         <v>26</v>
       </c>
@@ -2612,7 +2639,7 @@
       <c r="O39" s="3"/>
     </row>
     <row r="40" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="G40" s="50" t="s">
+      <c r="G40" s="45" t="s">
         <v>66</v>
       </c>
       <c r="H40" s="6" t="s">
@@ -2620,7 +2647,7 @@
       </c>
       <c r="I40" s="6"/>
       <c r="J40" s="7"/>
-      <c r="L40" s="46" t="s">
+      <c r="L40" s="44" t="s">
         <v>83</v>
       </c>
       <c r="M40" s="2" t="s">
@@ -2630,7 +2657,7 @@
       <c r="O40" s="3"/>
     </row>
     <row r="41" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B41" s="48" t="s">
+      <c r="B41" s="47" t="s">
         <v>33</v>
       </c>
       <c r="C41" s="11" t="s">
@@ -2640,7 +2667,7 @@
         <v>145</v>
       </c>
       <c r="E41" s="12"/>
-      <c r="G41" s="50"/>
+      <c r="G41" s="45"/>
       <c r="H41" s="2" t="s">
         <v>25</v>
       </c>
@@ -2648,7 +2675,7 @@
         <v>67</v>
       </c>
       <c r="J41" s="3"/>
-      <c r="L41" s="50"/>
+      <c r="L41" s="45"/>
       <c r="M41" s="2" t="s">
         <v>25</v>
       </c>
@@ -2656,7 +2683,7 @@
       <c r="O41" s="3"/>
     </row>
     <row r="42" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="50"/>
+      <c r="B42" s="45"/>
       <c r="C42" s="2" t="s">
         <v>25</v>
       </c>
@@ -2664,13 +2691,13 @@
         <v>11</v>
       </c>
       <c r="E42" s="3"/>
-      <c r="G42" s="49"/>
+      <c r="G42" s="46"/>
       <c r="H42" s="4" t="s">
         <v>26</v>
       </c>
       <c r="I42" s="4"/>
       <c r="J42" s="5"/>
-      <c r="L42" s="47"/>
+      <c r="L42" s="48"/>
       <c r="M42" s="2" t="s">
         <v>26</v>
       </c>
@@ -2678,7 +2705,7 @@
       <c r="O42" s="3"/>
     </row>
     <row r="43" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="47"/>
+      <c r="B43" s="48"/>
       <c r="C43" s="2" t="s">
         <v>26</v>
       </c>
@@ -2686,7 +2713,7 @@
         <v>11</v>
       </c>
       <c r="E43" s="3"/>
-      <c r="L43" s="46" t="s">
+      <c r="L43" s="44" t="s">
         <v>84</v>
       </c>
       <c r="M43" s="2" t="s">
@@ -2698,7 +2725,7 @@
       <c r="O43" s="3"/>
     </row>
     <row r="44" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B44" s="46" t="s">
+      <c r="B44" s="44" t="s">
         <v>34</v>
       </c>
       <c r="C44" s="2" t="s">
@@ -2706,7 +2733,7 @@
       </c>
       <c r="D44" s="2"/>
       <c r="E44" s="3"/>
-      <c r="G44" s="48" t="s">
+      <c r="G44" s="47" t="s">
         <v>68</v>
       </c>
       <c r="H44" s="11" t="s">
@@ -2716,7 +2743,7 @@
         <v>102</v>
       </c>
       <c r="J44" s="12"/>
-      <c r="L44" s="50"/>
+      <c r="L44" s="45"/>
       <c r="M44" s="2" t="s">
         <v>25</v>
       </c>
@@ -2728,7 +2755,7 @@
       </c>
     </row>
     <row r="45" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B45" s="50"/>
+      <c r="B45" s="45"/>
       <c r="C45" s="2" t="s">
         <v>25</v>
       </c>
@@ -2736,12 +2763,12 @@
         <v>12</v>
       </c>
       <c r="E45" s="3"/>
-      <c r="G45" s="50"/>
+      <c r="G45" s="45"/>
       <c r="H45" s="2" t="s">
         <v>25</v>
       </c>
       <c r="J45" s="3"/>
-      <c r="L45" s="47"/>
+      <c r="L45" s="48"/>
       <c r="M45" s="2" t="s">
         <v>26</v>
       </c>
@@ -2751,7 +2778,7 @@
       <c r="O45" s="3"/>
     </row>
     <row r="46" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B46" s="47"/>
+      <c r="B46" s="48"/>
       <c r="C46" s="2" t="s">
         <v>26</v>
       </c>
@@ -2759,7 +2786,7 @@
         <v>13</v>
       </c>
       <c r="E46" s="3"/>
-      <c r="G46" s="47"/>
+      <c r="G46" s="48"/>
       <c r="H46" s="2" t="s">
         <v>26</v>
       </c>
@@ -2769,7 +2796,7 @@
       <c r="J46" s="3" t="s">
         <v>170</v>
       </c>
-      <c r="L46" s="50" t="s">
+      <c r="L46" s="45" t="s">
         <v>183</v>
       </c>
       <c r="M46" s="2" t="s">
@@ -2779,7 +2806,7 @@
       <c r="O46" s="3"/>
     </row>
     <row r="47" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B47" s="46" t="s">
+      <c r="B47" s="44" t="s">
         <v>35</v>
       </c>
       <c r="C47" s="2" t="s">
@@ -2787,7 +2814,7 @@
       </c>
       <c r="D47" s="2"/>
       <c r="E47" s="3"/>
-      <c r="G47" s="46" t="s">
+      <c r="G47" s="44" t="s">
         <v>69</v>
       </c>
       <c r="H47" s="2" t="s">
@@ -2795,7 +2822,7 @@
       </c>
       <c r="I47" s="2"/>
       <c r="J47" s="3"/>
-      <c r="L47" s="50"/>
+      <c r="L47" s="45"/>
       <c r="M47" s="2" t="s">
         <v>25</v>
       </c>
@@ -2807,7 +2834,7 @@
       </c>
     </row>
     <row r="48" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B48" s="50"/>
+      <c r="B48" s="45"/>
       <c r="C48" s="2" t="s">
         <v>25</v>
       </c>
@@ -2815,13 +2842,13 @@
         <v>14</v>
       </c>
       <c r="E48" s="3"/>
-      <c r="G48" s="50"/>
+      <c r="G48" s="45"/>
       <c r="H48" s="2" t="s">
         <v>25</v>
       </c>
       <c r="I48" s="2"/>
       <c r="J48" s="3"/>
-      <c r="L48" s="49"/>
+      <c r="L48" s="46"/>
       <c r="M48" s="4" t="s">
         <v>26</v>
       </c>
@@ -2831,7 +2858,7 @@
       <c r="O48" s="5"/>
     </row>
     <row r="49" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B49" s="47"/>
+      <c r="B49" s="48"/>
       <c r="C49" s="2" t="s">
         <v>26</v>
       </c>
@@ -2839,7 +2866,7 @@
         <v>15</v>
       </c>
       <c r="E49" s="3"/>
-      <c r="G49" s="47"/>
+      <c r="G49" s="48"/>
       <c r="H49" s="2" t="s">
         <v>26</v>
       </c>
@@ -2847,7 +2874,7 @@
       <c r="J49" s="3"/>
     </row>
     <row r="50" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B50" s="46" t="s">
+      <c r="B50" s="44" t="s">
         <v>36</v>
       </c>
       <c r="C50" s="2" t="s">
@@ -2855,7 +2882,7 @@
       </c>
       <c r="D50" s="2"/>
       <c r="E50" s="3"/>
-      <c r="G50" s="46" t="s">
+      <c r="G50" s="44" t="s">
         <v>70</v>
       </c>
       <c r="H50" s="2" t="s">
@@ -2865,7 +2892,7 @@
         <v>103</v>
       </c>
       <c r="J50" s="3"/>
-      <c r="L50" s="48" t="s">
+      <c r="L50" s="47" t="s">
         <v>85</v>
       </c>
       <c r="M50" s="11" t="s">
@@ -2875,7 +2902,7 @@
       <c r="O50" s="12"/>
     </row>
     <row r="51" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B51" s="50"/>
+      <c r="B51" s="45"/>
       <c r="C51" s="2" t="s">
         <v>25</v>
       </c>
@@ -2883,12 +2910,12 @@
         <v>16</v>
       </c>
       <c r="E51" s="3"/>
-      <c r="G51" s="50"/>
+      <c r="G51" s="45"/>
       <c r="H51" s="2" t="s">
         <v>25</v>
       </c>
       <c r="J51" s="3"/>
-      <c r="L51" s="50"/>
+      <c r="L51" s="45"/>
       <c r="M51" s="2" t="s">
         <v>25</v>
       </c>
@@ -2898,7 +2925,7 @@
       <c r="O51" s="3"/>
     </row>
     <row r="52" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B52" s="49"/>
+      <c r="B52" s="46"/>
       <c r="C52" s="4" t="s">
         <v>26</v>
       </c>
@@ -2906,13 +2933,13 @@
         <v>17</v>
       </c>
       <c r="E52" s="5"/>
-      <c r="G52" s="49"/>
+      <c r="G52" s="46"/>
       <c r="H52" s="4" t="s">
         <v>26</v>
       </c>
       <c r="I52" s="4"/>
       <c r="J52" s="5"/>
-      <c r="L52" s="47"/>
+      <c r="L52" s="48"/>
       <c r="M52" s="2" t="s">
         <v>26</v>
       </c>
@@ -2920,7 +2947,7 @@
       <c r="O52" s="3"/>
     </row>
     <row r="53" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="L53" s="46" t="s">
+      <c r="L53" s="44" t="s">
         <v>86</v>
       </c>
       <c r="M53" s="2" t="s">
@@ -2930,7 +2957,7 @@
       <c r="O53" s="3"/>
     </row>
     <row r="54" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B54" s="48" t="s">
+      <c r="B54" s="47" t="s">
         <v>37</v>
       </c>
       <c r="C54" s="11" t="s">
@@ -2938,7 +2965,7 @@
       </c>
       <c r="D54" s="11"/>
       <c r="E54" s="12"/>
-      <c r="G54" s="48" t="s">
+      <c r="G54" s="47" t="s">
         <v>71</v>
       </c>
       <c r="H54" s="11" t="s">
@@ -2946,7 +2973,7 @@
       </c>
       <c r="I54" s="11"/>
       <c r="J54" s="12"/>
-      <c r="L54" s="50"/>
+      <c r="L54" s="45"/>
       <c r="M54" s="2" t="s">
         <v>25</v>
       </c>
@@ -2956,7 +2983,7 @@
       <c r="O54" s="3"/>
     </row>
     <row r="55" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B55" s="50"/>
+      <c r="B55" s="45"/>
       <c r="C55" s="2" t="s">
         <v>25</v>
       </c>
@@ -2964,7 +2991,7 @@
         <v>146</v>
       </c>
       <c r="E55" s="3"/>
-      <c r="G55" s="50"/>
+      <c r="G55" s="45"/>
       <c r="H55" s="2" t="s">
         <v>25</v>
       </c>
@@ -2972,7 +2999,7 @@
         <v>171</v>
       </c>
       <c r="J55" s="3"/>
-      <c r="L55" s="49"/>
+      <c r="L55" s="46"/>
       <c r="M55" s="4" t="s">
         <v>26</v>
       </c>
@@ -2980,13 +3007,13 @@
       <c r="O55" s="5"/>
     </row>
     <row r="56" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B56" s="47"/>
+      <c r="B56" s="48"/>
       <c r="C56" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D56" s="2"/>
       <c r="E56" s="3"/>
-      <c r="G56" s="47"/>
+      <c r="G56" s="48"/>
       <c r="H56" s="2" t="s">
         <v>26</v>
       </c>
@@ -2994,7 +3021,7 @@
       <c r="J56" s="3"/>
     </row>
     <row r="57" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B57" s="46" t="s">
+      <c r="B57" s="44" t="s">
         <v>38</v>
       </c>
       <c r="C57" s="2" t="s">
@@ -3002,7 +3029,7 @@
       </c>
       <c r="D57" s="2"/>
       <c r="E57" s="3"/>
-      <c r="G57" s="46" t="s">
+      <c r="G57" s="44" t="s">
         <v>72</v>
       </c>
       <c r="H57" s="2" t="s">
@@ -3010,7 +3037,7 @@
       </c>
       <c r="I57" s="2"/>
       <c r="J57" s="3"/>
-      <c r="L57" s="48" t="s">
+      <c r="L57" s="47" t="s">
         <v>87</v>
       </c>
       <c r="M57" s="11" t="s">
@@ -3020,7 +3047,7 @@
       <c r="O57" s="12"/>
     </row>
     <row r="58" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B58" s="50"/>
+      <c r="B58" s="45"/>
       <c r="C58" s="2" t="s">
         <v>25</v>
       </c>
@@ -3028,7 +3055,7 @@
         <v>147</v>
       </c>
       <c r="E58" s="3"/>
-      <c r="G58" s="50"/>
+      <c r="G58" s="45"/>
       <c r="H58" s="2" t="s">
         <v>25</v>
       </c>
@@ -3036,7 +3063,7 @@
         <v>172</v>
       </c>
       <c r="J58" s="3"/>
-      <c r="L58" s="50"/>
+      <c r="L58" s="45"/>
       <c r="M58" s="2" t="s">
         <v>25</v>
       </c>
@@ -3048,19 +3075,19 @@
       </c>
     </row>
     <row r="59" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B59" s="47"/>
+      <c r="B59" s="48"/>
       <c r="C59" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D59" s="2"/>
       <c r="E59" s="3"/>
-      <c r="G59" s="49"/>
+      <c r="G59" s="46"/>
       <c r="H59" s="4" t="s">
         <v>26</v>
       </c>
       <c r="I59" s="4"/>
       <c r="J59" s="5"/>
-      <c r="L59" s="47"/>
+      <c r="L59" s="48"/>
       <c r="M59" s="2" t="s">
         <v>26</v>
       </c>
@@ -3068,7 +3095,7 @@
       <c r="O59" s="3"/>
     </row>
     <row r="60" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B60" s="46" t="s">
+      <c r="B60" s="44" t="s">
         <v>39</v>
       </c>
       <c r="C60" s="2" t="s">
@@ -3076,7 +3103,7 @@
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="3"/>
-      <c r="L60" s="46" t="s">
+      <c r="L60" s="44" t="s">
         <v>88</v>
       </c>
       <c r="M60" s="2" t="s">
@@ -3086,7 +3113,7 @@
       <c r="O60" s="3"/>
     </row>
     <row r="61" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B61" s="50"/>
+      <c r="B61" s="45"/>
       <c r="C61" s="2" t="s">
         <v>25</v>
       </c>
@@ -3094,7 +3121,7 @@
         <v>148</v>
       </c>
       <c r="E61" s="3"/>
-      <c r="L61" s="50"/>
+      <c r="L61" s="45"/>
       <c r="M61" s="2" t="s">
         <v>25</v>
       </c>
@@ -3102,13 +3129,13 @@
       <c r="O61" s="3"/>
     </row>
     <row r="62" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B62" s="47"/>
+      <c r="B62" s="48"/>
       <c r="C62" s="2" t="s">
         <v>26</v>
       </c>
       <c r="D62" s="2"/>
       <c r="E62" s="3"/>
-      <c r="L62" s="47"/>
+      <c r="L62" s="48"/>
       <c r="M62" s="2" t="s">
         <v>26</v>
       </c>
@@ -3116,7 +3143,7 @@
       <c r="O62" s="3"/>
     </row>
     <row r="63" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B63" s="46" t="s">
+      <c r="B63" s="44" t="s">
         <v>40</v>
       </c>
       <c r="C63" s="2" t="s">
@@ -3124,7 +3151,7 @@
       </c>
       <c r="D63" s="2"/>
       <c r="E63" s="3"/>
-      <c r="L63" s="46" t="s">
+      <c r="L63" s="44" t="s">
         <v>89</v>
       </c>
       <c r="M63" s="2" t="s">
@@ -3134,7 +3161,7 @@
       <c r="O63" s="3"/>
     </row>
     <row r="64" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B64" s="50"/>
+      <c r="B64" s="45"/>
       <c r="C64" s="2" t="s">
         <v>25</v>
       </c>
@@ -3142,7 +3169,7 @@
         <v>149</v>
       </c>
       <c r="E64" s="3"/>
-      <c r="L64" s="50"/>
+      <c r="L64" s="45"/>
       <c r="M64" s="2" t="s">
         <v>25</v>
       </c>
@@ -3154,13 +3181,13 @@
       </c>
     </row>
     <row r="65" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B65" s="49"/>
+      <c r="B65" s="46"/>
       <c r="C65" s="4" t="s">
         <v>26</v>
       </c>
       <c r="D65" s="4"/>
       <c r="E65" s="5"/>
-      <c r="L65" s="47"/>
+      <c r="L65" s="48"/>
       <c r="M65" s="2" t="s">
         <v>26</v>
       </c>
@@ -3180,7 +3207,7 @@
       </c>
     </row>
     <row r="67" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B67" s="48" t="s">
+      <c r="B67" s="47" t="s">
         <v>41</v>
       </c>
       <c r="C67" s="11" t="s">
@@ -3194,7 +3221,7 @@
       </c>
     </row>
     <row r="68" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B68" s="50"/>
+      <c r="B68" s="45"/>
       <c r="C68" s="2" t="s">
         <v>25</v>
       </c>
@@ -3204,7 +3231,7 @@
       <c r="E68" s="3" t="s">
         <v>153</v>
       </c>
-      <c r="L68" s="48" t="s">
+      <c r="L68" s="47" t="s">
         <v>91</v>
       </c>
       <c r="M68" s="11" t="s">
@@ -3218,7 +3245,7 @@
       </c>
     </row>
     <row r="69" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B69" s="47"/>
+      <c r="B69" s="48"/>
       <c r="C69" s="2" t="s">
         <v>26</v>
       </c>
@@ -3226,7 +3253,7 @@
         <v>18</v>
       </c>
       <c r="E69" s="3"/>
-      <c r="L69" s="50"/>
+      <c r="L69" s="45"/>
       <c r="M69" s="2" t="s">
         <v>25</v>
       </c>
@@ -3238,7 +3265,7 @@
       </c>
     </row>
     <row r="70" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B70" s="46" t="s">
+      <c r="B70" s="44" t="s">
         <v>42</v>
       </c>
       <c r="C70" s="2" t="s">
@@ -3246,7 +3273,7 @@
       </c>
       <c r="D70" s="2"/>
       <c r="E70" s="3"/>
-      <c r="L70" s="47"/>
+      <c r="L70" s="48"/>
       <c r="M70" s="2" t="s">
         <v>26</v>
       </c>
@@ -3258,7 +3285,7 @@
       </c>
     </row>
     <row r="71" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B71" s="50"/>
+      <c r="B71" s="45"/>
       <c r="C71" s="2" t="s">
         <v>25</v>
       </c>
@@ -3266,7 +3293,7 @@
         <v>154</v>
       </c>
       <c r="E71" s="3"/>
-      <c r="L71" s="46" t="s">
+      <c r="L71" s="44" t="s">
         <v>92</v>
       </c>
       <c r="M71" s="2" t="s">
@@ -3276,7 +3303,7 @@
       <c r="O71" s="3"/>
     </row>
     <row r="72" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B72" s="47"/>
+      <c r="B72" s="48"/>
       <c r="C72" s="2" t="s">
         <v>26</v>
       </c>
@@ -3284,7 +3311,7 @@
         <v>19</v>
       </c>
       <c r="E72" s="3"/>
-      <c r="L72" s="50"/>
+      <c r="L72" s="45"/>
       <c r="M72" s="2" t="s">
         <v>25</v>
       </c>
@@ -3292,7 +3319,7 @@
       <c r="O72" s="3"/>
     </row>
     <row r="73" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B73" s="46" t="s">
+      <c r="B73" s="44" t="s">
         <v>43</v>
       </c>
       <c r="C73" s="2" t="s">
@@ -3300,7 +3327,7 @@
       </c>
       <c r="D73" s="2"/>
       <c r="E73" s="3"/>
-      <c r="L73" s="47"/>
+      <c r="L73" s="48"/>
       <c r="M73" s="2" t="s">
         <v>26</v>
       </c>
@@ -3308,7 +3335,7 @@
       <c r="O73" s="3"/>
     </row>
     <row r="74" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B74" s="50"/>
+      <c r="B74" s="45"/>
       <c r="C74" s="2" t="s">
         <v>25</v>
       </c>
@@ -3318,7 +3345,7 @@
       <c r="E74" s="3" t="s">
         <v>155</v>
       </c>
-      <c r="L74" s="46" t="s">
+      <c r="L74" s="44" t="s">
         <v>93</v>
       </c>
       <c r="M74" s="2" t="s">
@@ -3328,7 +3355,7 @@
       <c r="O74" s="3"/>
     </row>
     <row r="75" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B75" s="47"/>
+      <c r="B75" s="48"/>
       <c r="C75" s="2" t="s">
         <v>26</v>
       </c>
@@ -3336,7 +3363,7 @@
         <v>20</v>
       </c>
       <c r="E75" s="3"/>
-      <c r="L75" s="50"/>
+      <c r="L75" s="45"/>
       <c r="M75" s="2" t="s">
         <v>25</v>
       </c>
@@ -3348,7 +3375,7 @@
       </c>
     </row>
     <row r="76" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B76" s="46" t="s">
+      <c r="B76" s="44" t="s">
         <v>118</v>
       </c>
       <c r="C76" s="2" t="s">
@@ -3358,7 +3385,7 @@
         <v>0</v>
       </c>
       <c r="E76" s="3"/>
-      <c r="L76" s="49"/>
+      <c r="L76" s="46"/>
       <c r="M76" s="4" t="s">
         <v>26</v>
       </c>
@@ -3366,7 +3393,7 @@
       <c r="O76" s="5"/>
     </row>
     <row r="77" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B77" s="50"/>
+      <c r="B77" s="45"/>
       <c r="C77" s="2" t="s">
         <v>25</v>
       </c>
@@ -3378,7 +3405,7 @@
       </c>
     </row>
     <row r="78" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B78" s="47"/>
+      <c r="B78" s="48"/>
       <c r="C78" s="2" t="s">
         <v>26</v>
       </c>
@@ -3386,7 +3413,7 @@
         <v>0</v>
       </c>
       <c r="E78" s="3"/>
-      <c r="L78" s="48" t="s">
+      <c r="L78" s="47" t="s">
         <v>94</v>
       </c>
       <c r="M78" s="11" t="s">
@@ -3398,7 +3425,7 @@
       <c r="O78" s="12"/>
     </row>
     <row r="79" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B79" s="46" t="s">
+      <c r="B79" s="44" t="s">
         <v>44</v>
       </c>
       <c r="C79" s="2" t="s">
@@ -3406,7 +3433,7 @@
       </c>
       <c r="D79" s="2"/>
       <c r="E79" s="3"/>
-      <c r="L79" s="50"/>
+      <c r="L79" s="45"/>
       <c r="M79" s="2" t="s">
         <v>25</v>
       </c>
@@ -3418,7 +3445,7 @@
       </c>
     </row>
     <row r="80" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B80" s="50"/>
+      <c r="B80" s="45"/>
       <c r="C80" s="2" t="s">
         <v>25</v>
       </c>
@@ -3426,7 +3453,7 @@
         <v>157</v>
       </c>
       <c r="E80" s="3"/>
-      <c r="L80" s="47"/>
+      <c r="L80" s="48"/>
       <c r="M80" s="2" t="s">
         <v>26</v>
       </c>
@@ -3436,7 +3463,7 @@
       <c r="O80" s="3"/>
     </row>
     <row r="81" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B81" s="47"/>
+      <c r="B81" s="48"/>
       <c r="C81" s="2" t="s">
         <v>26</v>
       </c>
@@ -3444,7 +3471,7 @@
         <v>21</v>
       </c>
       <c r="E81" s="3"/>
-      <c r="L81" s="46" t="s">
+      <c r="L81" s="44" t="s">
         <v>95</v>
       </c>
       <c r="M81" s="2" t="s">
@@ -3454,7 +3481,7 @@
       <c r="O81" s="3"/>
     </row>
     <row r="82" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B82" s="46" t="s">
+      <c r="B82" s="44" t="s">
         <v>22</v>
       </c>
       <c r="C82" s="2" t="s">
@@ -3466,7 +3493,7 @@
       <c r="E82" s="3" t="s">
         <v>158</v>
       </c>
-      <c r="L82" s="50"/>
+      <c r="L82" s="45"/>
       <c r="M82" s="2" t="s">
         <v>25</v>
       </c>
@@ -3474,7 +3501,7 @@
       <c r="O82" s="3"/>
     </row>
     <row r="83" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B83" s="50"/>
+      <c r="B83" s="45"/>
       <c r="C83" s="2" t="s">
         <v>25</v>
       </c>
@@ -3484,7 +3511,7 @@
       <c r="E83" s="3" t="s">
         <v>159</v>
       </c>
-      <c r="L83" s="49"/>
+      <c r="L83" s="46"/>
       <c r="M83" s="4" t="s">
         <v>26</v>
       </c>
@@ -3492,7 +3519,7 @@
       <c r="O83" s="5"/>
     </row>
     <row r="84" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B84" s="49"/>
+      <c r="B84" s="46"/>
       <c r="C84" s="4" t="s">
         <v>26</v>
       </c>
@@ -3504,7 +3531,7 @@
       </c>
     </row>
     <row r="85" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="L85" s="48" t="s">
+      <c r="L85" s="47" t="s">
         <v>96</v>
       </c>
       <c r="M85" s="11" t="s">
@@ -3518,7 +3545,7 @@
       </c>
     </row>
     <row r="86" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="L86" s="50"/>
+      <c r="L86" s="45"/>
       <c r="M86" s="2" t="s">
         <v>25</v>
       </c>
@@ -3530,7 +3557,7 @@
       </c>
     </row>
     <row r="87" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="L87" s="47"/>
+      <c r="L87" s="48"/>
       <c r="M87" s="2" t="s">
         <v>26</v>
       </c>
@@ -3554,7 +3581,7 @@
       </c>
     </row>
     <row r="89" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="L89" s="46" t="s">
+      <c r="L89" s="44" t="s">
         <v>107</v>
       </c>
       <c r="M89" s="2" t="s">
@@ -3564,7 +3591,7 @@
       <c r="O89" s="3"/>
     </row>
     <row r="90" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="L90" s="50"/>
+      <c r="L90" s="45"/>
       <c r="M90" s="2" t="s">
         <v>25</v>
       </c>
@@ -3572,7 +3599,7 @@
       <c r="O90" s="3"/>
     </row>
     <row r="91" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="L91" s="49"/>
+      <c r="L91" s="46"/>
       <c r="M91" s="4" t="s">
         <v>26</v>
       </c>
@@ -3581,7 +3608,7 @@
     </row>
     <row r="92" spans="2:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="93" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="L93" s="48" t="s">
+      <c r="L93" s="47" t="s">
         <v>99</v>
       </c>
       <c r="M93" s="11" t="s">
@@ -3591,7 +3618,7 @@
       <c r="O93" s="12"/>
     </row>
     <row r="94" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="L94" s="50"/>
+      <c r="L94" s="45"/>
       <c r="M94" s="2" t="s">
         <v>25</v>
       </c>
@@ -3603,7 +3630,7 @@
       </c>
     </row>
     <row r="95" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="L95" s="47"/>
+      <c r="L95" s="48"/>
       <c r="M95" s="2" t="s">
         <v>26</v>
       </c>
@@ -3611,7 +3638,7 @@
       <c r="O95" s="3"/>
     </row>
     <row r="96" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="L96" s="46" t="s">
+      <c r="L96" s="44" t="s">
         <v>199</v>
       </c>
       <c r="M96" s="2" t="s">
@@ -3621,7 +3648,7 @@
       <c r="O96" s="3"/>
     </row>
     <row r="97" spans="12:15" x14ac:dyDescent="0.25">
-      <c r="L97" s="50"/>
+      <c r="L97" s="45"/>
       <c r="M97" s="2" t="s">
         <v>25</v>
       </c>
@@ -3633,7 +3660,7 @@
       </c>
     </row>
     <row r="98" spans="12:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="L98" s="49"/>
+      <c r="L98" s="46"/>
       <c r="M98" s="4" t="s">
         <v>26</v>
       </c>
@@ -3642,7 +3669,7 @@
     </row>
     <row r="99" spans="12:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="100" spans="12:15" x14ac:dyDescent="0.25">
-      <c r="L100" s="61" t="s">
+      <c r="L100" s="49" t="s">
         <v>97</v>
       </c>
       <c r="M100" s="38" t="s">
@@ -3652,7 +3679,7 @@
       <c r="O100" s="39"/>
     </row>
     <row r="101" spans="12:15" x14ac:dyDescent="0.25">
-      <c r="L101" s="62"/>
+      <c r="L101" s="50"/>
       <c r="M101" s="40" t="s">
         <v>25</v>
       </c>
@@ -3660,7 +3687,7 @@
       <c r="O101" s="41"/>
     </row>
     <row r="102" spans="12:15" x14ac:dyDescent="0.25">
-      <c r="L102" s="63"/>
+      <c r="L102" s="51"/>
       <c r="M102" s="40" t="s">
         <v>26</v>
       </c>
@@ -3668,7 +3695,7 @@
       <c r="O102" s="41"/>
     </row>
     <row r="103" spans="12:15" x14ac:dyDescent="0.25">
-      <c r="L103" s="64" t="s">
+      <c r="L103" s="52" t="s">
         <v>98</v>
       </c>
       <c r="M103" s="40" t="s">
@@ -3678,7 +3705,7 @@
       <c r="O103" s="41"/>
     </row>
     <row r="104" spans="12:15" x14ac:dyDescent="0.25">
-      <c r="L104" s="62"/>
+      <c r="L104" s="50"/>
       <c r="M104" s="40" t="s">
         <v>25</v>
       </c>
@@ -3686,7 +3713,7 @@
       <c r="O104" s="41"/>
     </row>
     <row r="105" spans="12:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="L105" s="65"/>
+      <c r="L105" s="53"/>
       <c r="M105" s="42" t="s">
         <v>26</v>
       </c>
@@ -3695,33 +3722,34 @@
     </row>
   </sheetData>
   <mergeCells count="71">
-    <mergeCell ref="L53:L55"/>
-    <mergeCell ref="L57:L59"/>
-    <mergeCell ref="L60:L62"/>
-    <mergeCell ref="L63:L65"/>
-    <mergeCell ref="L71:L73"/>
-    <mergeCell ref="L74:L76"/>
-    <mergeCell ref="L78:L80"/>
-    <mergeCell ref="L81:L83"/>
-    <mergeCell ref="L68:L70"/>
-    <mergeCell ref="L93:L95"/>
-    <mergeCell ref="L96:L98"/>
-    <mergeCell ref="L100:L102"/>
-    <mergeCell ref="L85:L87"/>
-    <mergeCell ref="L103:L105"/>
-    <mergeCell ref="L89:L91"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="G11:G13"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="L4:O4"/>
-    <mergeCell ref="G4:J4"/>
-    <mergeCell ref="B7:B9"/>
-    <mergeCell ref="L7:L8"/>
-    <mergeCell ref="L10:L11"/>
-    <mergeCell ref="L13:L14"/>
-    <mergeCell ref="L15:L17"/>
+    <mergeCell ref="J32:J33"/>
+    <mergeCell ref="G32:G33"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="L24:L26"/>
+    <mergeCell ref="L28:L29"/>
+    <mergeCell ref="L31:L32"/>
+    <mergeCell ref="L19:L23"/>
+    <mergeCell ref="L50:L52"/>
+    <mergeCell ref="L34:L36"/>
+    <mergeCell ref="L40:L42"/>
+    <mergeCell ref="L46:L48"/>
+    <mergeCell ref="L37:L39"/>
+    <mergeCell ref="L43:L45"/>
+    <mergeCell ref="G57:G59"/>
+    <mergeCell ref="B79:B81"/>
+    <mergeCell ref="G47:G49"/>
+    <mergeCell ref="G50:G52"/>
+    <mergeCell ref="B76:B78"/>
+    <mergeCell ref="B54:B56"/>
+    <mergeCell ref="G54:G56"/>
+    <mergeCell ref="G36:G38"/>
+    <mergeCell ref="B34:B36"/>
+    <mergeCell ref="B44:B46"/>
+    <mergeCell ref="B37:B39"/>
+    <mergeCell ref="B41:B43"/>
     <mergeCell ref="B82:B84"/>
     <mergeCell ref="B67:B69"/>
     <mergeCell ref="B70:B72"/>
@@ -3738,34 +3766,33 @@
     <mergeCell ref="B18:B20"/>
     <mergeCell ref="G40:G42"/>
     <mergeCell ref="G44:G46"/>
-    <mergeCell ref="G36:G38"/>
-    <mergeCell ref="B34:B36"/>
-    <mergeCell ref="B44:B46"/>
-    <mergeCell ref="B37:B39"/>
-    <mergeCell ref="B41:B43"/>
-    <mergeCell ref="G57:G59"/>
-    <mergeCell ref="B79:B81"/>
-    <mergeCell ref="G47:G49"/>
-    <mergeCell ref="G50:G52"/>
-    <mergeCell ref="B76:B78"/>
-    <mergeCell ref="B54:B56"/>
-    <mergeCell ref="G54:G56"/>
-    <mergeCell ref="L24:L26"/>
-    <mergeCell ref="L28:L29"/>
-    <mergeCell ref="L31:L32"/>
-    <mergeCell ref="L19:L23"/>
-    <mergeCell ref="L50:L52"/>
-    <mergeCell ref="L34:L36"/>
-    <mergeCell ref="L40:L42"/>
-    <mergeCell ref="L46:L48"/>
-    <mergeCell ref="L37:L39"/>
-    <mergeCell ref="L43:L45"/>
-    <mergeCell ref="J32:J33"/>
-    <mergeCell ref="G32:G33"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="G11:G13"/>
+    <mergeCell ref="B10:B12"/>
+    <mergeCell ref="B14:B16"/>
+    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="L4:O4"/>
+    <mergeCell ref="G4:J4"/>
+    <mergeCell ref="B7:B9"/>
+    <mergeCell ref="L7:L8"/>
+    <mergeCell ref="L10:L11"/>
+    <mergeCell ref="L13:L14"/>
+    <mergeCell ref="L15:L17"/>
+    <mergeCell ref="L96:L98"/>
+    <mergeCell ref="L100:L102"/>
+    <mergeCell ref="L85:L87"/>
+    <mergeCell ref="L103:L105"/>
+    <mergeCell ref="L89:L91"/>
+    <mergeCell ref="L74:L76"/>
+    <mergeCell ref="L78:L80"/>
+    <mergeCell ref="L81:L83"/>
+    <mergeCell ref="L68:L70"/>
+    <mergeCell ref="L93:L95"/>
+    <mergeCell ref="L53:L55"/>
+    <mergeCell ref="L57:L59"/>
+    <mergeCell ref="L60:L62"/>
+    <mergeCell ref="L63:L65"/>
+    <mergeCell ref="L71:L73"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="44" orientation="portrait" r:id="rId1"/>

</xml_diff>